<commit_message>
Add specialty columns to desk_assignments sample spreadsheet
Added "Specialty 1" and "Specialty 2" header columns after Desk Assignment,
with "Shipping and Delivery" (primary) and "Payments and Safety" (secondary)
populated in sample data rows. The upload service already parses these
columns: first specialty becomes primary, subsequent ones become secondary.

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,6 +435,80 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>Desk Assignment</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Specialty 1</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Specialty 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Jane Doe</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>jane.doe@example.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Support Desk</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Shipping and Delivery</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Payments and Safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>12346</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>John Smith</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>john.smith@example.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Support Desk</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Shipping and Delivery</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace & with and in Specialty 1 and Specialty 2 columns
https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -456,12 +456,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -490,12 +490,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -541,12 +541,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -558,12 +558,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -575,12 +575,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -626,12 +626,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -677,12 +677,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -711,12 +711,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -728,12 +728,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -745,12 +745,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -813,12 +813,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -847,12 +847,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -864,12 +864,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -898,12 +898,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -932,12 +932,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -966,12 +966,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1000,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1017,12 +1017,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1051,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1085,12 +1085,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1102,12 +1102,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1119,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1136,12 +1136,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1153,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1170,12 +1170,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1204,12 +1204,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1221,12 +1221,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1255,12 +1255,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1272,12 +1272,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1306,12 +1306,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1323,12 +1323,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -1374,12 +1374,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1476,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1493,12 +1493,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1510,12 +1510,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1527,12 +1527,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -1595,12 +1595,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -1714,12 +1714,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1731,12 +1731,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1765,12 +1765,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1833,12 +1833,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1850,12 +1850,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -1918,12 +1918,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1935,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1952,12 +1952,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1969,12 +1969,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1986,12 +1986,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2003,12 +2003,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2020,12 +2020,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2037,12 +2037,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2071,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2088,12 +2088,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2122,12 +2122,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2139,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2173,12 +2173,12 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2190,12 +2190,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2207,12 +2207,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2224,12 +2224,12 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2241,12 +2241,12 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2258,12 +2258,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2275,12 +2275,12 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2292,12 +2292,12 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2326,12 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2343,12 +2343,12 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2360,12 +2360,12 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2445,12 +2445,12 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2462,12 +2462,12 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2496,12 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2598,12 +2598,12 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2615,12 +2615,12 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2632,12 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2649,12 +2649,12 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2683,12 +2683,12 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2700,12 +2700,12 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2717,12 +2717,12 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2734,12 +2734,12 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2751,12 +2751,12 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2768,12 +2768,12 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2785,12 +2785,12 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2802,12 +2802,12 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2836,12 +2836,12 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2853,12 +2853,12 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2870,12 +2870,12 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -2904,12 +2904,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2938,12 +2938,12 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -3023,12 +3023,12 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -3057,12 +3057,12 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3091,12 +3091,12 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3108,12 +3108,12 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3125,12 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3142,12 +3142,12 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3159,12 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3193,12 +3193,12 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -3210,12 +3210,12 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -3244,12 +3244,12 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -3295,12 +3295,12 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -3380,12 +3380,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3397,12 +3397,12 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3414,12 +3414,12 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3448,12 +3448,12 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3465,12 +3465,12 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3482,12 +3482,12 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3499,12 +3499,12 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3516,12 +3516,12 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3533,12 +3533,12 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3550,12 +3550,12 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3567,12 +3567,12 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -3618,12 +3618,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3635,12 +3635,12 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -3686,12 +3686,12 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -3720,12 +3720,12 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3737,12 +3737,12 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3754,12 +3754,12 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3771,12 +3771,12 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3788,12 +3788,12 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3805,12 +3805,12 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -3839,12 +3839,12 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3856,12 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3873,12 +3873,12 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3890,12 +3890,12 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3907,12 +3907,12 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3924,12 +3924,12 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3941,12 +3941,12 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3958,12 +3958,12 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3975,12 +3975,12 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3992,12 +3992,12 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4009,12 +4009,12 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4026,12 +4026,12 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4043,12 +4043,12 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4060,12 +4060,12 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4077,12 +4077,12 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4111,12 +4111,12 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4128,12 +4128,12 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -4196,12 +4196,12 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
@@ -4247,12 +4247,12 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4264,12 +4264,12 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -4332,12 +4332,12 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4366,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -4383,12 +4383,12 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4400,12 +4400,12 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4417,12 +4417,12 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4434,12 +4434,12 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4451,12 +4451,12 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4468,12 +4468,12 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4485,12 +4485,12 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4502,12 +4502,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set Desk Assignment to EN I for all rows
https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -454,6 +454,11 @@
           <t>Anastasiia Sakharuk</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -471,6 +476,11 @@
           <t>Snizhana Zayats</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -488,6 +498,11 @@
           <t>Kateryna Podoliaka</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -505,6 +520,11 @@
           <t>Serhii Lutsenko</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -522,6 +542,11 @@
           <t>Mykhailo Cherepania</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -539,6 +564,11 @@
           <t>Tetiana Herman</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -556,6 +586,11 @@
           <t>Illia Makhniuk</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -573,6 +608,11 @@
           <t>Solomiia Krykhivska</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -590,6 +630,11 @@
           <t>Anastasiia Zaika</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -607,6 +652,11 @@
           <t>Anastasiia Zahoruiko</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -624,6 +674,11 @@
           <t>Nataliia Vonitova</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -641,6 +696,11 @@
           <t>Sesedzai Mudzingwa</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -658,6 +718,11 @@
           <t>Diana Khodan</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -675,6 +740,11 @@
           <t>Ihor Danyliak</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -692,6 +762,11 @@
           <t>Ashley Murerwa</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -709,6 +784,11 @@
           <t>Oleksii Pavlov</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -726,6 +806,11 @@
           <t>Yuliia Kravchuk</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -743,6 +828,11 @@
           <t>Ester Kovach</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -760,6 +850,11 @@
           <t>Anzhelika Kungurova</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -777,6 +872,11 @@
           <t>Dmytro Starozhytnyk</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -794,6 +894,11 @@
           <t>Nellia Kosenko</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -811,6 +916,11 @@
           <t>Andrii Abramov</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -828,6 +938,11 @@
           <t>Dmytro Lytvynenko</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -845,6 +960,11 @@
           <t>Tetiana Boiko</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -862,6 +982,11 @@
           <t>Vladyslav Vedmid</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -879,6 +1004,11 @@
           <t>Oleksii Komar</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -896,6 +1026,11 @@
           <t>Khrystyna Vyshnivska</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -913,6 +1048,11 @@
           <t>Anastasiia Solodka</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -930,6 +1070,11 @@
           <t>Yelyzaveta Tsyplenko</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -947,6 +1092,11 @@
           <t>Karina Pilipuitis</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -964,6 +1114,11 @@
           <t>Mariia Oros</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -981,6 +1136,11 @@
           <t>Oleksander Sviatchenko</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -998,6 +1158,11 @@
           <t>Anzhela Kulakova</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1015,6 +1180,11 @@
           <t>Bohdana Bohonos</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1032,6 +1202,11 @@
           <t>Vladyslav Kosovskyi</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1049,6 +1224,11 @@
           <t>Vladyslav Melnyk</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1066,6 +1246,11 @@
           <t>Tetiana Nazarenko</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1083,6 +1268,11 @@
           <t>Andrii Pryimenko</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1100,6 +1290,11 @@
           <t>Tetiana Kushnir</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1117,6 +1312,11 @@
           <t>Sofiia Maletska</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1134,6 +1334,11 @@
           <t>Andrii Manuliak</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1151,6 +1356,11 @@
           <t>Nataliia Trymbaliuk</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1168,6 +1378,11 @@
           <t>Sofiia Yukhymchuk</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1185,6 +1400,11 @@
           <t>Ilona Havryliuk</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1202,6 +1422,11 @@
           <t>Mariana Yuryshynets</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1219,6 +1444,11 @@
           <t>Anton Dmytruk</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1236,6 +1466,11 @@
           <t>Oleksandra Horobets</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1253,6 +1488,11 @@
           <t>Oleksandr Feshchuk</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1270,6 +1510,11 @@
           <t>Vitalii Yuzvyn</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1287,6 +1532,11 @@
           <t>Vladyslav Koreniuk</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1304,6 +1554,11 @@
           <t>Karolina-Anna Sikomas</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1321,6 +1576,11 @@
           <t>Dmytro Skrypak</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1338,6 +1598,11 @@
           <t>Yuliia Matviienko</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1355,6 +1620,11 @@
           <t>Mykola Sakalosh</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1372,6 +1642,11 @@
           <t>Hryhorii Balychev</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1389,6 +1664,11 @@
           <t>Bohdana Rudnevska</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1406,6 +1686,11 @@
           <t>Anastasiia Volkanova</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1423,6 +1708,11 @@
           <t>Olha Zubrytska</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1440,6 +1730,11 @@
           <t>Yevheniia Antonova</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1457,6 +1752,11 @@
           <t>Yekateryna Potsiluiko</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1474,6 +1774,11 @@
           <t>Andrii Venhreniuk</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -1491,6 +1796,11 @@
           <t>Yuliia Ruban</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1508,6 +1818,11 @@
           <t>Niiara Abdurakhmanova</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -1525,6 +1840,11 @@
           <t>Romanna Paniush</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -1542,6 +1862,11 @@
           <t>Borys Suiarko</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1559,6 +1884,11 @@
           <t>Bohdana Kosarchyn</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1576,6 +1906,11 @@
           <t>Kateryna Mazurenko</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1593,6 +1928,11 @@
           <t>Oladipo Rahmon Saliu</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1610,6 +1950,11 @@
           <t>Samuel Nwoke</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1627,6 +1972,11 @@
           <t>Anton Li</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1644,6 +1994,11 @@
           <t>Marina Pidkovenko</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1661,6 +2016,11 @@
           <t>Anton Dovhyi</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1678,6 +2038,11 @@
           <t>Vladyslav Melnychuk</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E74" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1695,6 +2060,11 @@
           <t>Olena Yaremenko1</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1712,6 +2082,11 @@
           <t>Sebastian Stroin</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1729,6 +2104,11 @@
           <t>Olena Sharlai</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1746,6 +2126,11 @@
           <t>Veronika Dzhaparidze</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1763,6 +2148,11 @@
           <t>Nataliia Karpiuk</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1780,6 +2170,11 @@
           <t>Sofia Hunka1</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1797,6 +2192,11 @@
           <t>Vadym Rakitin</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1814,6 +2214,11 @@
           <t>Serhii Koval</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1831,6 +2236,11 @@
           <t>Hlib Devecha</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1848,6 +2258,11 @@
           <t>Marta Chipko</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1865,6 +2280,11 @@
           <t>Korneliia Lopit</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1882,6 +2302,11 @@
           <t>Yuliia Udut</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1899,6 +2324,11 @@
           <t>Bohdan Dunaievskyi</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -1916,6 +2346,11 @@
           <t>Yevheniia Vlasenko</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1933,6 +2368,11 @@
           <t>Sofia Yurkiv</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1950,6 +2390,11 @@
           <t>Ivan Bekh</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1967,6 +2412,11 @@
           <t>Nazar-Marian Bakai</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1984,6 +2434,11 @@
           <t>Davyd Rozhkov</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2001,6 +2456,11 @@
           <t>Viktoriia Mysko</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2018,6 +2478,11 @@
           <t>Nazar Soloha</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2035,6 +2500,11 @@
           <t>Danil Diachenko</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2052,6 +2522,11 @@
           <t>Ihor Bohdan</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2069,6 +2544,11 @@
           <t>Mykhailo Shcherbyna</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2086,6 +2566,11 @@
           <t>Anastasiia Vynnyk</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2103,6 +2588,11 @@
           <t>Asan Khalilov</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2120,6 +2610,11 @@
           <t>Tetiana Krat</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2137,6 +2632,11 @@
           <t>Marharyta Kohut</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2154,6 +2654,11 @@
           <t>Yana Kovalenko</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2171,6 +2676,11 @@
           <t>Yelyzaveta Nadieieva</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2188,6 +2698,11 @@
           <t>Maksym Patrai</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2205,6 +2720,11 @@
           <t>Khrystyna Pelyno</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2222,6 +2742,11 @@
           <t>Mariia Tarasiuk</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2239,6 +2764,11 @@
           <t>Valentyna Vanzuriak</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2256,6 +2786,11 @@
           <t>Khrystyna Koprovska</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2273,6 +2808,11 @@
           <t>Yevhen Kushnyrik</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E109" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2290,6 +2830,11 @@
           <t>Maksym Kukharyk</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E110" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2307,6 +2852,11 @@
           <t>Danylo Hushcha</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2324,6 +2874,11 @@
           <t>Karolina Onyshchenko</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E112" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2341,6 +2896,11 @@
           <t>Yurii Sosnovskyi</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E113" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2358,6 +2918,11 @@
           <t>Vladyslav Tiutiunnyk</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2375,6 +2940,11 @@
           <t>Danyil Muravlov</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2392,6 +2962,11 @@
           <t>Anna Korkeshko</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E116" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2409,6 +2984,11 @@
           <t>Andriana Budysh</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2426,6 +3006,11 @@
           <t>Widgen Ropafadzo Tsabora</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E118" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2443,6 +3028,11 @@
           <t>Kamilla Kukri</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2460,6 +3050,11 @@
           <t>Sviatoslav Mezhivnyk</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E120" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2477,6 +3072,11 @@
           <t>Daryna Stankevych</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2494,6 +3094,11 @@
           <t>Marta Smuk</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2511,6 +3116,11 @@
           <t>Volodymyr Koziupa</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2528,6 +3138,11 @@
           <t>Oleksii Petrov</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2545,6 +3160,11 @@
           <t>Mariia Popova</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2562,6 +3182,11 @@
           <t>Yevheniia Prokopiv</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2579,6 +3204,11 @@
           <t>Valentyna Bulik</t>
         </is>
       </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2596,6 +3226,11 @@
           <t>Oksana Nykoliak</t>
         </is>
       </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2613,6 +3248,11 @@
           <t>Olena Dymura</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2630,6 +3270,11 @@
           <t>Yevheniia Vakulina</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2647,6 +3292,11 @@
           <t>Kateryna Dzyha</t>
         </is>
       </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2664,6 +3314,11 @@
           <t>Roman Sivak</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2681,6 +3336,11 @@
           <t>Orest Labiak</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2698,6 +3358,11 @@
           <t>Kostiantyn Pinchuk</t>
         </is>
       </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E134" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2715,6 +3380,11 @@
           <t>Anna Pozniak</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E135" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2732,6 +3402,11 @@
           <t>Anna Shumyk</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2749,6 +3424,11 @@
           <t>Anastasiia Lavryk</t>
         </is>
       </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E137" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2766,6 +3446,11 @@
           <t>Bogdan Ryabenko</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E138" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2783,6 +3468,11 @@
           <t>Vladyslava Zharska</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E139" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2800,6 +3490,11 @@
           <t>Dmytro Tkachenko</t>
         </is>
       </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E140" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2817,6 +3512,11 @@
           <t>Yelyzaveta Bozhko</t>
         </is>
       </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E141" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2834,6 +3534,11 @@
           <t>Olha Yaroshenko</t>
         </is>
       </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E142" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2851,6 +3556,11 @@
           <t>Kostiantyn Pohrebniak</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2868,6 +3578,11 @@
           <t>Denys Lebeda</t>
         </is>
       </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2885,6 +3600,11 @@
           <t>Yuliia Zhygulina</t>
         </is>
       </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E145" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2902,6 +3622,11 @@
           <t>Diana Rudzik</t>
         </is>
       </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E146" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2919,6 +3644,11 @@
           <t>Yakiv Kysliakov</t>
         </is>
       </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2936,6 +3666,11 @@
           <t>Nazar Drahomirov</t>
         </is>
       </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E148" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2953,6 +3688,11 @@
           <t>Volodymyr Larin</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E149" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2970,6 +3710,11 @@
           <t>Mariia Boncheva</t>
         </is>
       </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E150" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -2987,6 +3732,11 @@
           <t>Maksym Orlov1</t>
         </is>
       </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E151" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3004,6 +3754,11 @@
           <t>Mykhailo Senychych</t>
         </is>
       </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E152" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3021,6 +3776,11 @@
           <t>Yevhen Kelembet</t>
         </is>
       </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3038,6 +3798,11 @@
           <t>Volodymyr Larin</t>
         </is>
       </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E154" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3055,6 +3820,11 @@
           <t>Ihor Klimenchenko</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E155" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3072,6 +3842,11 @@
           <t>Maryna Polishchuk</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3089,6 +3864,11 @@
           <t>Anastasiia Kozbur</t>
         </is>
       </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E157" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3106,6 +3886,11 @@
           <t>Oleksandr Mykolaiko</t>
         </is>
       </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E158" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3123,6 +3908,11 @@
           <t>Valeriia Makovetska</t>
         </is>
       </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3140,6 +3930,11 @@
           <t>Olena Matviiv</t>
         </is>
       </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E160" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3157,6 +3952,11 @@
           <t>Maksym Kulish</t>
         </is>
       </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E161" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3174,6 +3974,11 @@
           <t>Victoria Kushnir</t>
         </is>
       </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E162" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3191,6 +3996,11 @@
           <t>Aleksandra Kvitka</t>
         </is>
       </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E163" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3208,6 +4018,11 @@
           <t>Mohamad Kawni</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3225,6 +4040,11 @@
           <t>Maryna Kibak</t>
         </is>
       </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E165" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3242,6 +4062,11 @@
           <t>Victoria Petrova</t>
         </is>
       </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3259,6 +4084,11 @@
           <t>Mykhailo Zelenchuk</t>
         </is>
       </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3276,6 +4106,11 @@
           <t>Mariia Shapovalenko</t>
         </is>
       </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3293,6 +4128,11 @@
           <t>Vladyslav Hoza</t>
         </is>
       </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3310,6 +4150,11 @@
           <t>Markiian Hanushevskyi</t>
         </is>
       </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3327,6 +4172,11 @@
           <t>Artem Sehal</t>
         </is>
       </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E171" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3344,6 +4194,11 @@
           <t>Ilona Ilieva</t>
         </is>
       </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3361,6 +4216,11 @@
           <t>Makar Bytsyura</t>
         </is>
       </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E173" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3378,6 +4238,11 @@
           <t>Taras Tiurdo</t>
         </is>
       </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E174" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3395,6 +4260,11 @@
           <t>Danylo Honchar</t>
         </is>
       </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3412,6 +4282,11 @@
           <t>Ivan Horobets</t>
         </is>
       </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E176" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3429,6 +4304,11 @@
           <t>Illia Yaremenko</t>
         </is>
       </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E177" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3446,6 +4326,11 @@
           <t>Anastasiia Ratushna</t>
         </is>
       </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E178" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3463,6 +4348,11 @@
           <t>Daniil Komiakov</t>
         </is>
       </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E179" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3480,6 +4370,11 @@
           <t>Denys Fedchenko</t>
         </is>
       </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E180" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3497,6 +4392,11 @@
           <t>Olesia Kuzyk</t>
         </is>
       </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E181" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3514,6 +4414,11 @@
           <t>Anastasiya Skibynska</t>
         </is>
       </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E182" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3531,6 +4436,11 @@
           <t>Ivan Kravchenko</t>
         </is>
       </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E183" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3548,6 +4458,11 @@
           <t>Valerii Zaiarnyi</t>
         </is>
       </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E184" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3565,6 +4480,11 @@
           <t>Viktoriia Avramenko</t>
         </is>
       </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E185" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3582,6 +4502,11 @@
           <t>Anhelina Turianska</t>
         </is>
       </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E186" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3599,6 +4524,11 @@
           <t>Olena Halaktionova</t>
         </is>
       </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E187" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3616,6 +4546,11 @@
           <t>Vitalii Radchenko</t>
         </is>
       </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E188" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3633,6 +4568,11 @@
           <t>Petro Fenenko</t>
         </is>
       </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E189" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3650,6 +4590,11 @@
           <t>Yevhen Fedorchenko</t>
         </is>
       </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E190" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3667,6 +4612,11 @@
           <t>Sofiia Zaianchkivska</t>
         </is>
       </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E191" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3684,6 +4634,11 @@
           <t>Oleksandr Matviichuk</t>
         </is>
       </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E192" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3701,6 +4656,11 @@
           <t>Valerii Toderiuk</t>
         </is>
       </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3718,6 +4678,11 @@
           <t>Mariana Humeniuk</t>
         </is>
       </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E194" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3735,6 +4700,11 @@
           <t>Viktor Lyulka</t>
         </is>
       </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E195" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3752,6 +4722,11 @@
           <t>Liudmyla Plekhanova</t>
         </is>
       </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E196" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3769,6 +4744,11 @@
           <t>Yehor Keller</t>
         </is>
       </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E197" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3786,6 +4766,11 @@
           <t>Dmytro Suprunets</t>
         </is>
       </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E198" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3803,6 +4788,11 @@
           <t>Viktor Dunets</t>
         </is>
       </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E199" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3820,6 +4810,11 @@
           <t>Nikita Havryliuk</t>
         </is>
       </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E200" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -3837,6 +4832,11 @@
           <t>Yuliia Bosko</t>
         </is>
       </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E201" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3854,6 +4854,11 @@
           <t>Alona Dehtiar</t>
         </is>
       </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E202" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3871,6 +4876,11 @@
           <t>Alina Nikolaieva</t>
         </is>
       </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E203" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3888,6 +4898,11 @@
           <t>Anastasiia Zykova</t>
         </is>
       </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E204" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3905,6 +4920,11 @@
           <t>Maksym Olynets</t>
         </is>
       </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E205" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3922,6 +4942,11 @@
           <t>Oleksandr Prepiialo</t>
         </is>
       </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E206" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3939,6 +4964,11 @@
           <t>Vadym Kharchenko</t>
         </is>
       </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E207" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3956,6 +4986,11 @@
           <t>Nikol Benua Berko</t>
         </is>
       </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E208" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3973,6 +5008,11 @@
           <t>Dmytro Mitsiuk</t>
         </is>
       </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E209" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3990,6 +5030,11 @@
           <t>Eduard Nesterenko</t>
         </is>
       </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E210" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4007,6 +5052,11 @@
           <t>Mariia Bodak</t>
         </is>
       </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E211" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4024,6 +5074,11 @@
           <t>Vitalii Marchenko</t>
         </is>
       </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E212" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4041,6 +5096,11 @@
           <t>Kostiantyn Bratchenko</t>
         </is>
       </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E213" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4058,6 +5118,11 @@
           <t>Romana Hrynovets</t>
         </is>
       </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E214" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4075,6 +5140,11 @@
           <t>Olha Prymak</t>
         </is>
       </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E215" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4092,6 +5162,11 @@
           <t>Veronika Bondar</t>
         </is>
       </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E216" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4109,6 +5184,11 @@
           <t>Nika Karpinska</t>
         </is>
       </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E217" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4126,6 +5206,11 @@
           <t>Valeriia Sereda</t>
         </is>
       </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E218" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4143,6 +5228,11 @@
           <t>Taras Tatarskyi</t>
         </is>
       </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E219" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4160,6 +5250,11 @@
           <t>Danylo Zhurniev</t>
         </is>
       </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E220" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4177,6 +5272,11 @@
           <t>Sofiia Bilyk</t>
         </is>
       </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E221" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4194,6 +5294,11 @@
           <t>Yuliia Hlynska</t>
         </is>
       </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E222" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4211,6 +5316,11 @@
           <t>Roman Zavhorodnii</t>
         </is>
       </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E223" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4228,6 +5338,11 @@
           <t>Artem Stratonov</t>
         </is>
       </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E224" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4245,6 +5360,11 @@
           <t>Denys Pronkin</t>
         </is>
       </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E225" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -4262,6 +5382,11 @@
           <t>Valerii Pylypenko</t>
         </is>
       </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E226" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4279,6 +5404,11 @@
           <t>Kateryna Lohin</t>
         </is>
       </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E227" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4296,6 +5426,11 @@
           <t>Arsen Shkolnyi</t>
         </is>
       </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E228" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4313,6 +5448,11 @@
           <t>Melusi Karen Kombore</t>
         </is>
       </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4330,6 +5470,11 @@
           <t>Kateryna Vasylovych</t>
         </is>
       </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E230" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4347,6 +5492,11 @@
           <t>Lolita Liushyn</t>
         </is>
       </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4364,6 +5514,11 @@
           <t>Alyona Zalevska</t>
         </is>
       </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E232" t="inlineStr">
         <is>
           <t>Privacy and Legal</t>
@@ -4381,6 +5536,11 @@
           <t>Iryna Tsolta</t>
         </is>
       </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E233" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4398,6 +5558,11 @@
           <t>Mykyta Koval</t>
         </is>
       </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E234" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -4415,6 +5580,11 @@
           <t>Sofiia Komziuk</t>
         </is>
       </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E235" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4432,6 +5602,11 @@
           <t>Dmytro Chaievskyi</t>
         </is>
       </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E236" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4449,6 +5624,11 @@
           <t>Diana Rykhalska</t>
         </is>
       </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E237" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4466,6 +5646,11 @@
           <t>Oleh Metlenko</t>
         </is>
       </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E238" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4483,6 +5668,11 @@
           <t>Maksym Starominskyi</t>
         </is>
       </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E239" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -4498,6 +5688,11 @@
       <c r="B240" t="inlineStr">
         <is>
           <t>Denys Hohol</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>EN I</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">

</xml_diff>

<commit_message>
Rename "Payments and Safety" to "Payments and Safety & DSA" in desk assignments spreadsheet
Updated 60 cells across Specialty 1 and Specialty 2 columns.

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -483,7 +483,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -505,7 +505,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5565,7 +5565,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Payments and Safety</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">

</xml_diff>

<commit_message>
Rename "DSA" to "Payments and Safety & DSA" in desk assignments spreadsheet
Updated 51 cells across Specialty 1 and Specialty 2 columns.

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -664,7 +664,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5460,7 +5460,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Payments and Safety &amp; DSA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace ampersands with "and" in desk_assignments spreadsheet
Updated all 427 cells containing "&" to use "and" instead across
the desk_assignments.xlsx file (e.g., "Payments & Safety" -> "Payments and Safety").

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -456,12 +456,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -490,12 +490,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -541,12 +541,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -558,12 +558,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -575,12 +575,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -626,12 +626,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -677,12 +677,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -711,12 +711,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -728,12 +728,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -745,12 +745,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -813,12 +813,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -847,12 +847,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -864,12 +864,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -898,12 +898,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -932,12 +932,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -966,12 +966,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1000,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1017,12 +1017,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1051,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1085,12 +1085,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1102,12 +1102,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1119,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1136,12 +1136,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1153,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1170,12 +1170,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1204,12 +1204,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1221,12 +1221,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1255,12 +1255,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1272,12 +1272,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1306,12 +1306,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1323,12 +1323,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -1374,12 +1374,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1476,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1493,12 +1493,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1510,12 +1510,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1527,12 +1527,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -1595,12 +1595,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -1714,12 +1714,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1731,12 +1731,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1765,12 +1765,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1833,12 +1833,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1850,12 +1850,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -1918,12 +1918,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1935,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -1952,12 +1952,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1969,12 +1969,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -1986,12 +1986,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2003,12 +2003,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2020,12 +2020,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2037,12 +2037,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2071,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2088,12 +2088,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2122,12 +2122,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2139,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2173,12 +2173,12 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2190,12 +2190,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2207,12 +2207,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2224,12 +2224,12 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2241,12 +2241,12 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2258,12 +2258,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2275,12 +2275,12 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2292,12 +2292,12 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2326,12 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2343,12 +2343,12 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2360,12 +2360,12 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2445,12 +2445,12 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2462,12 +2462,12 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2496,12 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2598,12 +2598,12 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2615,12 +2615,12 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2632,12 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2649,12 +2649,12 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2683,12 +2683,12 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2700,12 +2700,12 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2717,12 +2717,12 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2734,12 +2734,12 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2751,12 +2751,12 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2768,12 +2768,12 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2785,12 +2785,12 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2802,12 +2802,12 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2836,12 +2836,12 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -2853,12 +2853,12 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2870,12 +2870,12 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -2904,12 +2904,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -2938,12 +2938,12 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -3023,12 +3023,12 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -3057,12 +3057,12 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3091,12 +3091,12 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3108,12 +3108,12 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3125,12 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3142,12 +3142,12 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3159,12 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3193,12 +3193,12 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -3210,12 +3210,12 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -3244,12 +3244,12 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -3295,12 +3295,12 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -3380,12 +3380,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3397,12 +3397,12 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3414,12 +3414,12 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3448,12 +3448,12 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3465,12 +3465,12 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3482,12 +3482,12 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3499,12 +3499,12 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3516,12 +3516,12 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3533,12 +3533,12 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3550,12 +3550,12 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3567,12 +3567,12 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -3618,12 +3618,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3635,12 +3635,12 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -3686,12 +3686,12 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -3720,12 +3720,12 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3737,12 +3737,12 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3754,12 +3754,12 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3771,12 +3771,12 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -3788,12 +3788,12 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3805,12 +3805,12 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -3839,12 +3839,12 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3856,12 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3873,12 +3873,12 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3890,12 +3890,12 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3907,12 +3907,12 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3924,12 +3924,12 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3941,12 +3941,12 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3958,12 +3958,12 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3975,12 +3975,12 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -3992,12 +3992,12 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4009,12 +4009,12 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4026,12 +4026,12 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4043,12 +4043,12 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4060,12 +4060,12 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4077,12 +4077,12 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4111,12 +4111,12 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4128,12 +4128,12 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -4196,12 +4196,12 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
@@ -4247,12 +4247,12 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4264,12 +4264,12 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -4332,12 +4332,12 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4366,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Privacy &amp; Legal</t>
+          <t>Privacy and Legal</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -4383,12 +4383,12 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4400,12 +4400,12 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4417,12 +4417,12 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4434,12 +4434,12 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4451,12 +4451,12 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>
@@ -4468,12 +4468,12 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4485,12 +4485,12 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Payments &amp; Safety</t>
+          <t>Payments and Safety</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
     </row>
@@ -4502,12 +4502,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Shipping &amp; Delivery</t>
+          <t>Shipping and Delivery</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Order Quality &amp; Usability</t>
+          <t>Order Quality and Usability</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace "Privacy and Legal" and "DSA" with "Privacy and Legal & DSA" in desk_assignments
Updated 102 cells in Specialty 1 and Specialty 2 columns to consolidate
"Privacy and Legal" and "DSA" into the single value "Privacy and Legal & DSA".

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -609,12 +609,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -643,12 +643,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -660,12 +660,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -796,12 +796,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1340,12 +1340,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1357,12 +1357,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1425,12 +1425,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1442,12 +1442,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1561,12 +1561,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1578,12 +1578,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1612,12 +1612,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1629,12 +1629,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1663,12 +1663,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1782,12 +1782,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2377,12 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2394,12 +2394,12 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2411,12 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2513,12 +2513,12 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2530,12 +2530,12 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2887,12 +2887,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2972,12 +2972,12 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3006,12 +3006,12 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3040,12 +3040,12 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3227,12 +3227,12 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3261,12 +3261,12 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3278,12 +3278,12 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3312,12 +3312,12 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3346,12 +3346,12 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3601,12 +3601,12 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3652,12 +3652,12 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3669,12 +3669,12 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3703,12 +3703,12 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -3822,12 +3822,12 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4162,12 +4162,12 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4179,12 +4179,12 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4213,12 +4213,12 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4230,12 +4230,12 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4281,12 +4281,12 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4298,12 +4298,12 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4315,12 +4315,12 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>
@@ -4366,12 +4366,12 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Privacy and Legal</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Privacy and Legal &amp; DSA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set all Desk Assignment values to "EN I" in desk_assignments spreadsheet
Updated 239 cells in the Desk Assignment column to "EN I".

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/desk_assignments.xlsx
+++ b/src/main/resources/sample-data/desk_assignments.xlsx
@@ -454,6 +454,11 @@
           <t>Anastasiia Sakharuk</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -471,6 +476,11 @@
           <t>Snizhana Zayats</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -488,6 +498,11 @@
           <t>Kateryna Podoliaka</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -505,6 +520,11 @@
           <t>Serhii Lutsenko</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -522,6 +542,11 @@
           <t>Mykhailo Cherepania</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -539,6 +564,11 @@
           <t>Tetiana Herman</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -556,6 +586,11 @@
           <t>Illia Makhniuk</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -573,6 +608,11 @@
           <t>Solomiia Krykhivska</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -590,6 +630,11 @@
           <t>Anastasiia Zaika</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -607,6 +652,11 @@
           <t>Anastasiia Zahoruiko</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -624,6 +674,11 @@
           <t>Nataliia Vonitova</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -641,6 +696,11 @@
           <t>Sesedzai Mudzingwa</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -658,6 +718,11 @@
           <t>Diana Khodan</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -675,6 +740,11 @@
           <t>Ihor Danyliak</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -692,6 +762,11 @@
           <t>Ashley Murerwa</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -709,6 +784,11 @@
           <t>Oleksii Pavlov</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -726,6 +806,11 @@
           <t>Yuliia Kravchuk</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -743,6 +828,11 @@
           <t>Ester Kovach</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -760,6 +850,11 @@
           <t>Anzhelika Kungurova</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -777,6 +872,11 @@
           <t>Dmytro Starozhytnyk</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -794,6 +894,11 @@
           <t>Nellia Kosenko</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -811,6 +916,11 @@
           <t>Andrii Abramov</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -828,6 +938,11 @@
           <t>Dmytro Lytvynenko</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -845,6 +960,11 @@
           <t>Tetiana Boiko</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -862,6 +982,11 @@
           <t>Vladyslav Vedmid</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -879,6 +1004,11 @@
           <t>Oleksii Komar</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -896,6 +1026,11 @@
           <t>Khrystyna Vyshnivska</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -913,6 +1048,11 @@
           <t>Anastasiia Solodka</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -930,6 +1070,11 @@
           <t>Yelyzaveta Tsyplenko</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -947,6 +1092,11 @@
           <t>Karina Pilipuitis</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -964,6 +1114,11 @@
           <t>Mariia Oros</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -981,6 +1136,11 @@
           <t>Oleksander Sviatchenko</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -998,6 +1158,11 @@
           <t>Anzhela Kulakova</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1015,6 +1180,11 @@
           <t>Bohdana Bohonos</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1032,6 +1202,11 @@
           <t>Vladyslav Kosovskyi</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1049,6 +1224,11 @@
           <t>Vladyslav Melnyk</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1066,6 +1246,11 @@
           <t>Tetiana Nazarenko</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1083,6 +1268,11 @@
           <t>Andrii Pryimenko</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1100,6 +1290,11 @@
           <t>Tetiana Kushnir</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1117,6 +1312,11 @@
           <t>Sofiia Maletska</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1134,6 +1334,11 @@
           <t>Andrii Manuliak</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1151,6 +1356,11 @@
           <t>Nataliia Trymbaliuk</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1168,6 +1378,11 @@
           <t>Sofiia Yukhymchuk</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1185,6 +1400,11 @@
           <t>Ilona Havryliuk</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1202,6 +1422,11 @@
           <t>Mariana Yuryshynets</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1219,6 +1444,11 @@
           <t>Anton Dmytruk</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1236,6 +1466,11 @@
           <t>Oleksandra Horobets</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1253,6 +1488,11 @@
           <t>Oleksandr Feshchuk</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1270,6 +1510,11 @@
           <t>Vitalii Yuzvyn</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1287,6 +1532,11 @@
           <t>Vladyslav Koreniuk</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1304,6 +1554,11 @@
           <t>Karolina-Anna Sikomas</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1321,6 +1576,11 @@
           <t>Dmytro Skrypak</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1338,6 +1598,11 @@
           <t>Yuliia Matviienko</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1355,6 +1620,11 @@
           <t>Mykola Sakalosh</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1372,6 +1642,11 @@
           <t>Hryhorii Balychev</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1389,6 +1664,11 @@
           <t>Bohdana Rudnevska</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1406,6 +1686,11 @@
           <t>Anastasiia Volkanova</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1423,6 +1708,11 @@
           <t>Olha Zubrytska</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1440,6 +1730,11 @@
           <t>Yevheniia Antonova</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1457,6 +1752,11 @@
           <t>Yekateryna Potsiluiko</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1474,6 +1774,11 @@
           <t>Andrii Venhreniuk</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -1491,6 +1796,11 @@
           <t>Yuliia Ruban</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1508,6 +1818,11 @@
           <t>Niiara Abdurakhmanova</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -1525,6 +1840,11 @@
           <t>Romanna Paniush</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -1542,6 +1862,11 @@
           <t>Borys Suiarko</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1559,6 +1884,11 @@
           <t>Bohdana Kosarchyn</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1576,6 +1906,11 @@
           <t>Kateryna Mazurenko</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1593,6 +1928,11 @@
           <t>Oladipo Rahmon Saliu</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1610,6 +1950,11 @@
           <t>Samuel Nwoke</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1627,6 +1972,11 @@
           <t>Anton Li</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1644,6 +1994,11 @@
           <t>Marina Pidkovenko</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1661,6 +2016,11 @@
           <t>Anton Dovhyi</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1678,6 +2038,11 @@
           <t>Vladyslav Melnychuk</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E74" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1695,6 +2060,11 @@
           <t>Olena Yaremenko1</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1712,6 +2082,11 @@
           <t>Sebastian Stroin</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1729,6 +2104,11 @@
           <t>Olena Sharlai</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1746,6 +2126,11 @@
           <t>Veronika Dzhaparidze</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1763,6 +2148,11 @@
           <t>Nataliia Karpiuk</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1780,6 +2170,11 @@
           <t>Sofia Hunka1</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1797,6 +2192,11 @@
           <t>Vadym Rakitin</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1814,6 +2214,11 @@
           <t>Serhii Koval</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1831,6 +2236,11 @@
           <t>Hlib Devecha</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1848,6 +2258,11 @@
           <t>Marta Chipko</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1865,6 +2280,11 @@
           <t>Korneliia Lopit</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1882,6 +2302,11 @@
           <t>Yuliia Udut</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1899,6 +2324,11 @@
           <t>Bohdan Dunaievskyi</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -1916,6 +2346,11 @@
           <t>Yevheniia Vlasenko</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1933,6 +2368,11 @@
           <t>Sofia Yurkiv</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -1950,6 +2390,11 @@
           <t>Ivan Bekh</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1967,6 +2412,11 @@
           <t>Nazar-Marian Bakai</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -1984,6 +2434,11 @@
           <t>Davyd Rozhkov</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2001,6 +2456,11 @@
           <t>Viktoriia Mysko</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2018,6 +2478,11 @@
           <t>Nazar Soloha</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2035,6 +2500,11 @@
           <t>Danil Diachenko</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2052,6 +2522,11 @@
           <t>Ihor Bohdan</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2069,6 +2544,11 @@
           <t>Mykhailo Shcherbyna</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2086,6 +2566,11 @@
           <t>Anastasiia Vynnyk</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2103,6 +2588,11 @@
           <t>Asan Khalilov</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2120,6 +2610,11 @@
           <t>Tetiana Krat</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2137,6 +2632,11 @@
           <t>Marharyta Kohut</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2154,6 +2654,11 @@
           <t>Yana Kovalenko</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2171,6 +2676,11 @@
           <t>Yelyzaveta Nadieieva</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2188,6 +2698,11 @@
           <t>Maksym Patrai</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2205,6 +2720,11 @@
           <t>Khrystyna Pelyno</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2222,6 +2742,11 @@
           <t>Mariia Tarasiuk</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2239,6 +2764,11 @@
           <t>Valentyna Vanzuriak</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2256,6 +2786,11 @@
           <t>Khrystyna Koprovska</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2273,6 +2808,11 @@
           <t>Yevhen Kushnyrik</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E109" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2290,6 +2830,11 @@
           <t>Maksym Kukharyk</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E110" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2307,6 +2852,11 @@
           <t>Danylo Hushcha</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2324,6 +2874,11 @@
           <t>Karolina Onyshchenko</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E112" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2341,6 +2896,11 @@
           <t>Yurii Sosnovskyi</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E113" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2358,6 +2918,11 @@
           <t>Vladyslav Tiutiunnyk</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2375,6 +2940,11 @@
           <t>Danyil Muravlov</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2392,6 +2962,11 @@
           <t>Anna Korkeshko</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E116" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2409,6 +2984,11 @@
           <t>Andriana Budysh</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2426,6 +3006,11 @@
           <t>Widgen Ropafadzo Tsabora</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E118" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2443,6 +3028,11 @@
           <t>Kamilla Kukri</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2460,6 +3050,11 @@
           <t>Sviatoslav Mezhivnyk</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E120" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2477,6 +3072,11 @@
           <t>Daryna Stankevych</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2494,6 +3094,11 @@
           <t>Marta Smuk</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2511,6 +3116,11 @@
           <t>Volodymyr Koziupa</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2528,6 +3138,11 @@
           <t>Oleksii Petrov</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2545,6 +3160,11 @@
           <t>Mariia Popova</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2562,6 +3182,11 @@
           <t>Yevheniia Prokopiv</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2579,6 +3204,11 @@
           <t>Valentyna Bulik</t>
         </is>
       </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2596,6 +3226,11 @@
           <t>Oksana Nykoliak</t>
         </is>
       </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2613,6 +3248,11 @@
           <t>Olena Dymura</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2630,6 +3270,11 @@
           <t>Yevheniia Vakulina</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2647,6 +3292,11 @@
           <t>Kateryna Dzyha</t>
         </is>
       </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2664,6 +3314,11 @@
           <t>Roman Sivak</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2681,6 +3336,11 @@
           <t>Orest Labiak</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2698,6 +3358,11 @@
           <t>Kostiantyn Pinchuk</t>
         </is>
       </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E134" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2715,6 +3380,11 @@
           <t>Anna Pozniak</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E135" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2732,6 +3402,11 @@
           <t>Anna Shumyk</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2749,6 +3424,11 @@
           <t>Anastasiia Lavryk</t>
         </is>
       </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E137" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2766,6 +3446,11 @@
           <t>Bogdan Ryabenko</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E138" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2783,6 +3468,11 @@
           <t>Vladyslava Zharska</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E139" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2800,6 +3490,11 @@
           <t>Dmytro Tkachenko</t>
         </is>
       </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E140" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2817,6 +3512,11 @@
           <t>Yelyzaveta Bozhko</t>
         </is>
       </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E141" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2834,6 +3534,11 @@
           <t>Olha Yaroshenko</t>
         </is>
       </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E142" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2851,6 +3556,11 @@
           <t>Kostiantyn Pohrebniak</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2868,6 +3578,11 @@
           <t>Denys Lebeda</t>
         </is>
       </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -2885,6 +3600,11 @@
           <t>Yuliia Zhygulina</t>
         </is>
       </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E145" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2902,6 +3622,11 @@
           <t>Diana Rudzik</t>
         </is>
       </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E146" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2919,6 +3644,11 @@
           <t>Yakiv Kysliakov</t>
         </is>
       </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -2936,6 +3666,11 @@
           <t>Nazar Drahomirov</t>
         </is>
       </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E148" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -2953,6 +3688,11 @@
           <t>Volodymyr Larin</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E149" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2970,6 +3710,11 @@
           <t>Mariia Boncheva</t>
         </is>
       </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E150" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -2987,6 +3732,11 @@
           <t>Maksym Orlov1</t>
         </is>
       </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E151" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3004,6 +3754,11 @@
           <t>Mykhailo Senychych</t>
         </is>
       </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E152" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3021,6 +3776,11 @@
           <t>Yevhen Kelembet</t>
         </is>
       </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3038,6 +3798,11 @@
           <t>Volodymyr Larin</t>
         </is>
       </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E154" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3055,6 +3820,11 @@
           <t>Ihor Klimenchenko</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E155" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3072,6 +3842,11 @@
           <t>Maryna Polishchuk</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3089,6 +3864,11 @@
           <t>Anastasiia Kozbur</t>
         </is>
       </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E157" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3106,6 +3886,11 @@
           <t>Oleksandr Mykolaiko</t>
         </is>
       </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E158" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3123,6 +3908,11 @@
           <t>Valeriia Makovetska</t>
         </is>
       </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3140,6 +3930,11 @@
           <t>Olena Matviiv</t>
         </is>
       </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E160" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3157,6 +3952,11 @@
           <t>Maksym Kulish</t>
         </is>
       </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E161" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3174,6 +3974,11 @@
           <t>Victoria Kushnir</t>
         </is>
       </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E162" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3191,6 +3996,11 @@
           <t>Aleksandra Kvitka</t>
         </is>
       </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E163" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3208,6 +4018,11 @@
           <t>Mohamad Kawni</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3225,6 +4040,11 @@
           <t>Maryna Kibak</t>
         </is>
       </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E165" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3242,6 +4062,11 @@
           <t>Victoria Petrova</t>
         </is>
       </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3259,6 +4084,11 @@
           <t>Mykhailo Zelenchuk</t>
         </is>
       </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3276,6 +4106,11 @@
           <t>Mariia Shapovalenko</t>
         </is>
       </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3293,6 +4128,11 @@
           <t>Vladyslav Hoza</t>
         </is>
       </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3310,6 +4150,11 @@
           <t>Markiian Hanushevskyi</t>
         </is>
       </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3327,6 +4172,11 @@
           <t>Artem Sehal</t>
         </is>
       </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E171" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3344,6 +4194,11 @@
           <t>Ilona Ilieva</t>
         </is>
       </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3361,6 +4216,11 @@
           <t>Makar Bytsyura</t>
         </is>
       </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E173" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3378,6 +4238,11 @@
           <t>Taras Tiurdo</t>
         </is>
       </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E174" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3395,6 +4260,11 @@
           <t>Danylo Honchar</t>
         </is>
       </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3412,6 +4282,11 @@
           <t>Ivan Horobets</t>
         </is>
       </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E176" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3429,6 +4304,11 @@
           <t>Illia Yaremenko</t>
         </is>
       </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E177" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3446,6 +4326,11 @@
           <t>Anastasiia Ratushna</t>
         </is>
       </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E178" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3463,6 +4348,11 @@
           <t>Daniil Komiakov</t>
         </is>
       </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E179" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3480,6 +4370,11 @@
           <t>Denys Fedchenko</t>
         </is>
       </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E180" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3497,6 +4392,11 @@
           <t>Olesia Kuzyk</t>
         </is>
       </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E181" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3514,6 +4414,11 @@
           <t>Anastasiya Skibynska</t>
         </is>
       </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E182" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3531,6 +4436,11 @@
           <t>Ivan Kravchenko</t>
         </is>
       </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E183" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3548,6 +4458,11 @@
           <t>Valerii Zaiarnyi</t>
         </is>
       </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E184" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3565,6 +4480,11 @@
           <t>Viktoriia Avramenko</t>
         </is>
       </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E185" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3582,6 +4502,11 @@
           <t>Anhelina Turianska</t>
         </is>
       </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E186" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3599,6 +4524,11 @@
           <t>Olena Halaktionova</t>
         </is>
       </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E187" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3616,6 +4546,11 @@
           <t>Vitalii Radchenko</t>
         </is>
       </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E188" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3633,6 +4568,11 @@
           <t>Petro Fenenko</t>
         </is>
       </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E189" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -3650,6 +4590,11 @@
           <t>Yevhen Fedorchenko</t>
         </is>
       </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E190" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3667,6 +4612,11 @@
           <t>Sofiia Zaianchkivska</t>
         </is>
       </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E191" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3684,6 +4634,11 @@
           <t>Oleksandr Matviichuk</t>
         </is>
       </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E192" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3701,6 +4656,11 @@
           <t>Valerii Toderiuk</t>
         </is>
       </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3718,6 +4678,11 @@
           <t>Mariana Humeniuk</t>
         </is>
       </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E194" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3735,6 +4700,11 @@
           <t>Viktor Lyulka</t>
         </is>
       </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E195" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3752,6 +4722,11 @@
           <t>Liudmyla Plekhanova</t>
         </is>
       </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E196" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3769,6 +4744,11 @@
           <t>Yehor Keller</t>
         </is>
       </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E197" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -3786,6 +4766,11 @@
           <t>Dmytro Suprunets</t>
         </is>
       </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E198" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3803,6 +4788,11 @@
           <t>Viktor Dunets</t>
         </is>
       </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E199" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3820,6 +4810,11 @@
           <t>Nikita Havryliuk</t>
         </is>
       </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E200" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -3837,6 +4832,11 @@
           <t>Yuliia Bosko</t>
         </is>
       </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E201" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3854,6 +4854,11 @@
           <t>Alona Dehtiar</t>
         </is>
       </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E202" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3871,6 +4876,11 @@
           <t>Alina Nikolaieva</t>
         </is>
       </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E203" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3888,6 +4898,11 @@
           <t>Anastasiia Zykova</t>
         </is>
       </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E204" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3905,6 +4920,11 @@
           <t>Maksym Olynets</t>
         </is>
       </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E205" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3922,6 +4942,11 @@
           <t>Oleksandr Prepiialo</t>
         </is>
       </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E206" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3939,6 +4964,11 @@
           <t>Vadym Kharchenko</t>
         </is>
       </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E207" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3956,6 +4986,11 @@
           <t>Nikol Benua Berko</t>
         </is>
       </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E208" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3973,6 +5008,11 @@
           <t>Dmytro Mitsiuk</t>
         </is>
       </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E209" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -3990,6 +5030,11 @@
           <t>Eduard Nesterenko</t>
         </is>
       </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E210" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4007,6 +5052,11 @@
           <t>Mariia Bodak</t>
         </is>
       </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E211" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4024,6 +5074,11 @@
           <t>Vitalii Marchenko</t>
         </is>
       </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E212" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4041,6 +5096,11 @@
           <t>Kostiantyn Bratchenko</t>
         </is>
       </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E213" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4058,6 +5118,11 @@
           <t>Romana Hrynovets</t>
         </is>
       </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E214" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4075,6 +5140,11 @@
           <t>Olha Prymak</t>
         </is>
       </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E215" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4092,6 +5162,11 @@
           <t>Veronika Bondar</t>
         </is>
       </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E216" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4109,6 +5184,11 @@
           <t>Nika Karpinska</t>
         </is>
       </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E217" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4126,6 +5206,11 @@
           <t>Valeriia Sereda</t>
         </is>
       </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E218" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4143,6 +5228,11 @@
           <t>Taras Tatarskyi</t>
         </is>
       </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E219" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4160,6 +5250,11 @@
           <t>Danylo Zhurniev</t>
         </is>
       </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E220" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4177,6 +5272,11 @@
           <t>Sofiia Bilyk</t>
         </is>
       </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E221" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4194,6 +5294,11 @@
           <t>Yuliia Hlynska</t>
         </is>
       </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E222" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4211,6 +5316,11 @@
           <t>Roman Zavhorodnii</t>
         </is>
       </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E223" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4228,6 +5338,11 @@
           <t>Artem Stratonov</t>
         </is>
       </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E224" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4245,6 +5360,11 @@
           <t>Denys Pronkin</t>
         </is>
       </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E225" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -4262,6 +5382,11 @@
           <t>Valerii Pylypenko</t>
         </is>
       </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E226" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4279,6 +5404,11 @@
           <t>Kateryna Lohin</t>
         </is>
       </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E227" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4296,6 +5426,11 @@
           <t>Arsen Shkolnyi</t>
         </is>
       </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E228" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4313,6 +5448,11 @@
           <t>Melusi Karen Kombore</t>
         </is>
       </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4330,6 +5470,11 @@
           <t>Kateryna Vasylovych</t>
         </is>
       </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E230" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4347,6 +5492,11 @@
           <t>Lolita Liushyn</t>
         </is>
       </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4364,6 +5514,11 @@
           <t>Alyona Zalevska</t>
         </is>
       </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E232" t="inlineStr">
         <is>
           <t>Privacy and Legal &amp; DSA</t>
@@ -4381,6 +5536,11 @@
           <t>Iryna Tsolta</t>
         </is>
       </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E233" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4398,6 +5558,11 @@
           <t>Mykyta Koval</t>
         </is>
       </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E234" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -4415,6 +5580,11 @@
           <t>Sofiia Komziuk</t>
         </is>
       </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E235" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4432,6 +5602,11 @@
           <t>Dmytro Chaievskyi</t>
         </is>
       </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E236" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4449,6 +5624,11 @@
           <t>Diana Rykhalska</t>
         </is>
       </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E237" t="inlineStr">
         <is>
           <t>Shipping and Delivery</t>
@@ -4466,6 +5646,11 @@
           <t>Oleh Metlenko</t>
         </is>
       </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E238" t="inlineStr">
         <is>
           <t>Order Quality and Usability</t>
@@ -4483,6 +5668,11 @@
           <t>Maksym Starominskyi</t>
         </is>
       </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>EN I</t>
+        </is>
+      </c>
       <c r="E239" t="inlineStr">
         <is>
           <t>Payments and Safety</t>
@@ -4498,6 +5688,11 @@
       <c r="B240" t="inlineStr">
         <is>
           <t>Denys Hohol</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>EN I</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">

</xml_diff>